<commit_message>
Update COT classifications: DOC, PLA GEN, PLA DET, REU INT, REU CTTAL, VIS
- DOC = 40 UF, PLA DET = 25 UF, PLA GEN = 20 UF
- REU INT = 1 UF, REU CTTAL = 1 UF, VIS = 25 UF
- Updated template Excel with new types and examples
- Updated pricing logic in COT preview and totals

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/matriz-intranet/public/Cotizacion_Plantilla.xlsx
+++ b/matriz-intranet/public/Cotizacion_Plantilla.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -514,7 +514,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>CRD</t>
+          <t>DOC</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -537,7 +537,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>EETT</t>
+          <t>DOC</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -560,17 +560,17 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>MTO</t>
+          <t>PLA GEN</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Memoria Técnica</t>
+          <t>Planta General</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Memoria de Cálculo Obras Civiles</t>
+          <t>Planta de Disposición General - Nivel 1</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
@@ -583,7 +583,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>PLA DET</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -606,21 +606,21 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>GRL</t>
+          <t>REU INT</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Planta General</t>
+          <t>Reunión Interna</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Planta de Cielos y Luminarias</t>
+          <t>Reunión de coordinación interna equipo</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="7">
@@ -629,21 +629,44 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>REU CTTAL</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Detalle de Instalación</t>
+          <t>Reunión Contractual</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Detalle de Montaje Estructura Metálica</t>
+          <t>Reunión con mandante revisión avance</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>VIS</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Visita a Terreno</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Visita de inspección a faena</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -658,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -739,102 +762,109 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  CRD (Criterios de Diseño)  →  40 UF por unidad</t>
+          <t xml:space="preserve">  DOC (Documento técnico)  →  40 UF por unidad</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EETT (Especificaciones Técnicas)  →  40 UF por unidad</t>
+          <t xml:space="preserve">  PLA GEN (Plano General)  →  20 UF por unidad</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MTO (Memoria Técnica / Cálculo)  →  40 UF por unidad</t>
+          <t xml:space="preserve">  PLA DET (Plano de Detalle)  →  25 UF por unidad</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DET (Detalle Constructivo)  →  25 UF por unidad</t>
+          <t xml:space="preserve">  REU INT (Reunión Interna)  →  1 UF por unidad</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  GRL (General / Otros)  →  20 UF por unidad</t>
+          <t xml:space="preserve">  REU CTTAL (Reunión Contractual)  →  1 UF por unidad</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  VIS (Visita a Terreno)  →  25 UF por unidad</t>
+        </is>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+      <c r="A19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
         <is>
           <t>DISTRIBUCIÓN DE PAGOS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  REV_A  →  70% del total (entrega)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  REV_B  →  20% del total (con observaciones)</t>
+          <t xml:space="preserve">  REV_A  →  70% del total (entrega)</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  REV_B  →  20% del total (con observaciones)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">  REV_0  →  10% del total (aprobación final)</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr"/>
-    </row>
     <row r="24">
-      <c r="A24" s="6" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>NOTAS:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - Elimine las filas de ejemplo antes de completar sus datos.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Solo se procesan filas que tengan DESCRIPCIÓN (columna D).</t>
+          <t xml:space="preserve">  - Elimine las filas de ejemplo antes de completar sus datos.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  - Si no indica CLASIFICACIÓN, se asume GRL (20 UF).</t>
+          <t xml:space="preserve">  - Solo se procesan filas que tengan DESCRIPCIÓN (columna D).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - Si no indica CLASIFICACIÓN, se asume PLA GEN (20 UF).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">  - Si no indica CANTIDAD, se asume 1.</t>
         </is>

</xml_diff>